<commit_message>
feat: implement bulk upload service updates for new question types and add supporting Excel templates with documentation.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_contact_details_upload.xlsx
+++ b/frontend/public/templates/sample_contact_details_upload.xlsx
@@ -54,19 +54,30 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,21 +444,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,60 +524,302 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>http://sample.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sample Org</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>123 Main St</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Seattle</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>98101</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>206-555-0199</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>info@sample.com</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://facebook.com/sampleorg</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://globalcorp1.net</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Global Corp 1 Solutions</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Suite 100, Corporate Tower</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>022-2266-0001</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>support@globalcorp1.net</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/globalcorp1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_CONTACT_DETAILS</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>FRESHER</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://globalcorp2.net</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Global Corp 2 Solutions</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Suite 200, Corporate Tower</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>022-2266-0002</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>support@globalcorp2.net</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/globalcorp2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_CONTACT_DETAILS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FRESHER</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://globalcorp3.net</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Global Corp 3 Solutions</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Suite 300, Corporate Tower</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>022-2266-0003</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>support@globalcorp3.net</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/globalcorp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_CONTACT_DETAILS</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>FRESHER</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://globalcorp4.net</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Global Corp 4 Solutions</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Suite 400, Corporate Tower</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>022-2266-0004</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>support@globalcorp4.net</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/globalcorp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_CONTACT_DETAILS</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>FRESHER</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://globalcorp5.net</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Global Corp 5 Solutions</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Suite 500, Corporate Tower</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>400001</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>022-2266-0005</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>support@globalcorp5.net</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/globalcorp5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update sample data upload templates to current specifications
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_contact_details_upload.xlsx
+++ b/frontend/public/templates/sample_contact_details_upload.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,19 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF333333"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,8 +55,13 @@
         <bgColor rgb="00f96331"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF96331"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -67,16 +83,57 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -444,380 +501,391 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Question Id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Subject Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Exam Level Code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Marks</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Website URL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Organization</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Street Address</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Zip Code</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Facebook Page</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="D2" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>https://globalcorp1.net</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Global Corp 1 Solutions</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Suite 100, Corporate Tower</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>400001</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>022-2266-0001</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>support@globalcorp1.net</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>https://facebook.com/globalcorp1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="D3" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>https://globalcorp2.net</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Global Corp 2 Solutions</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Suite 200, Corporate Tower</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>400001</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>022-2266-0002</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>support@globalcorp2.net</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>https://facebook.com/globalcorp2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="D4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>https://globalcorp3.net</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Global Corp 3 Solutions</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Suite 300, Corporate Tower</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>400001</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>022-2266-0003</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>support@globalcorp3.net</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>https://facebook.com/globalcorp3</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="D5" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>https://globalcorp4.net</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Global Corp 4 Solutions</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Suite 400, Corporate Tower</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>400001</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>022-2266-0004</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>support@globalcorp4.net</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>https://facebook.com/globalcorp4</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>COMPANY_CONTACT_DETAILS</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>FRESHER</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="D6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>https://globalcorp5.net</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Global Corp 5 Solutions</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Suite 500, Corporate Tower</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>400001</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>022-2266-0005</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>support@globalcorp5.net</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>https://facebook.com/globalcorp5</t>
         </is>

</xml_diff>